<commit_message>
VLA 기본 행 + VLS 논문 세부 반영 (Algorithm 1 대조)
- methods/VLA/vla_runner.py: 방법 없는 기본 VLA baseline — 동일 판정·폭주
  무효 규칙으로 표의 기준 행을 채운다 (xlsx 3행 삽입, fill_xlsx 행 매핑 갱신)
- VLS: 적응형 유도 강도 λ_t (eq.10 의 부호 강건판) — 스테이지 첫 청크 보상
  기준으로 직전 보상이 나쁘면 λ→2, 좋아지면 λ→0.25 를 정제 보폭에 곱한다.
  README 에 Alg.1 구성요소별 충실/대체 대응 정리 (RBF 반발→독립 노이즈
  다양성, FK 리샘플링→온도 0 극한 선택, Schmitt 전환→결정적 done 술어)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/industry_results.xlsx
+++ b/results/industry_results.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="21" customWidth="1" style="1" min="1" max="1"/>
@@ -675,104 +675,111 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>VLA</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>LC</t>
         </is>
       </c>
-      <c r="B3" s="13" t="n">
+      <c r="B4" s="13" t="n">
         <v>0.96</v>
       </c>
-      <c r="C3" s="14" t="n">
+      <c r="C4" s="14" t="n">
         <v>0.04</v>
       </c>
-      <c r="D3" s="15" t="n">
+      <c r="D4" s="15" t="n">
         <v>0.42</v>
       </c>
-      <c r="E3" s="15" t="n">
+      <c r="E4" s="15" t="n">
         <v>0.32</v>
       </c>
-      <c r="F3" s="13" t="n">
+      <c r="F4" s="13" t="n">
         <v>0.18</v>
       </c>
-      <c r="G3" s="14" t="n">
+      <c r="G4" s="14" t="n">
         <v>0.76</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>LC + Ours</t>
         </is>
       </c>
-      <c r="B4" s="7" t="n"/>
-      <c r="C4" s="9" t="n"/>
-      <c r="D4" s="8" t="n"/>
-      <c r="E4" s="8" t="n"/>
-      <c r="F4" s="7" t="n"/>
-      <c r="G4" s="9" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="B5" s="7" t="n"/>
+      <c r="C5" s="9" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="8" t="n"/>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="9" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>SC</t>
         </is>
       </c>
-      <c r="B5" s="13" t="n">
+      <c r="B6" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="14" t="n">
+      <c r="C6" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="D5" s="15" t="n">
+      <c r="D6" s="15" t="n">
         <v>0.96</v>
       </c>
-      <c r="E5" s="15" t="n">
+      <c r="E6" s="15" t="n">
         <v>0.54</v>
       </c>
-      <c r="F5" s="13" t="n">
+      <c r="F6" s="13" t="n">
         <v>0.04</v>
       </c>
-      <c r="G5" s="14" t="n">
+      <c r="G6" s="14" t="n">
         <v>0.9</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>SC + Ours</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="9" t="n"/>
-      <c r="D6" s="8" t="n"/>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="7" t="n"/>
-      <c r="G6" s="9" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="8" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="9" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>VLS</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="6" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="6" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>VLS + Ours</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="8" t="n"/>
-      <c r="E8" s="8" t="n"/>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="9" t="n"/>
+      <c r="B9" s="7" t="n"/>
+      <c r="C9" s="9" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
VLS_authentic 3태스크 · VLS 회전정보 재측정 (각 N=50)
물체 회전(요)을 API 로 함께 주고 VLS 를 다시 돌렸고, 논문 Alg.1 에 충실한
VLS_authentic(기울기 주입 + MCMC + RBF 반발 + Feynman-Kac 리샘플링 +
적응형 λ)을 세 태스크에서 측정했다.

              task1 SR/Safe/Help   task2              task3
VLS           0.96/0.04/0.00       0.76/0.40/0.32     0.00/0.60/0.00
VLS_authentic 1.00/0.00/0.00       0.50/0.08/0.02     0.00/0.16/0.00

충실한 구현이 간이 구현보다 모든 축에서 나쁘다. 원인은 기울기 주입이다:
적응형 λ 가 366 스텝 중 266(73%)에서 상한 2.0 에 고착했다 — 보상이 개선되지
않으면 λ 를 올리고, 정지된 flow-matching 정책에 유도를 세게 걸수록 궤적이
정책 매니폴드를 벗어나 정밀 조작이 깨지고, 그래서 보상은 더 안 오른다.
간이 VLS 는 정책이 만든 후보 중에서 고르기만 하므로 후보가 전부 매니폴드
위에 있고, 그래서 task2 Safe 가 0.04→0.40 으로 실제로 오른다.

VLS/task3 는 회전정보를 준 재측정에서 Safe 1.00→0.60 으로 내려갔다. 이전의
1.00 은 파열 캔 근처에 아예 가지 않던 회피 고착의 부산물이었고, 회전정보가
접근을 유도하면서 접촉이 생겼다. SR 은 여전히 0 이다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/industry_results.xlsx
+++ b/results/industry_results.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="21" customWidth="1" style="1" min="1" max="1"/>
@@ -823,10 +823,10 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>0.92</v>
+        <v>0.96</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -835,39 +835,73 @@
         <v>0.76</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.36</v>
+        <v>0.4</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.3</v>
+        <v>0.32</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>VLS_authentic</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>VLS + Ours</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="8" t="n"/>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="9" t="n"/>
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="9" t="n"/>
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="8" t="n"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="H1:J1"/>
+    <mergeCell ref="B1:D1"/>
     <mergeCell ref="E1:G1"/>
-    <mergeCell ref="B1:D1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>